<commit_message>
sheet update Harshidha Narendran
</commit_message>
<xml_diff>
--- a/scripts/files/COCO AU SHEET 16926.xlsx
+++ b/scripts/files/COCO AU SHEET 16926.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30611"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{587E2A93-2720-4B35-B7DE-B04CD48769AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{33995A95-B65A-47D6-8ED6-078CA2226CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Property Name</t>
   </si>
@@ -45,7 +45,7 @@
     <t>SYSTEM ROOM NO</t>
   </si>
   <si>
-    <t>Coco Living AU</t>
+    <t>Coco | Au</t>
   </si>
 </sst>
 </file>
@@ -426,56 +426,23 @@
         <v>4</v>
       </c>
       <c r="B2" s="2">
-        <v>9112683627</v>
+        <v>7358241985</v>
       </c>
       <c r="C2">
-        <v>511</v>
+        <v>204</v>
       </c>
       <c r="D2">
-        <v>512</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="20.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2">
-        <v>8669994544</v>
-      </c>
-      <c r="C3">
-        <v>512</v>
-      </c>
-      <c r="D3">
-        <v>511</v>
-      </c>
+      <c r="B3" s="2"/>
     </row>
     <row r="4" spans="1:4" ht="20.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2">
-        <v>9022586799</v>
-      </c>
-      <c r="C4">
-        <v>402</v>
-      </c>
-      <c r="D4">
-        <v>204</v>
-      </c>
+      <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="20.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2">
-        <v>7358241985</v>
-      </c>
-      <c r="C5">
-        <v>204</v>
-      </c>
-      <c r="D5">
-        <v>402</v>
-      </c>
+      <c r="B5" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>